<commit_message>
Refactor indentation logic (#120)
</commit_message>
<xml_diff>
--- a/tests/data/dat.xlsx
+++ b/tests/data/dat.xlsx
@@ -22,16 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,26 +420,31 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.2" customWidth="1" min="1" max="1"/>
+    <col width="13.2" customWidth="1" min="2" max="2"/>
+    <col width="13.2" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -464,7 +457,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -477,7 +470,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -490,7 +483,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -515,31 +508,38 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.1" customWidth="1" min="1" max="1"/>
+    <col width="13.2" customWidth="1" min="2" max="2"/>
+    <col width="13.2" customWidth="1" min="3" max="3"/>
+    <col width="13.2" customWidth="1" min="4" max="4"/>
+    <col width="13.2" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -558,7 +558,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
@@ -591,24 +591,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -621,7 +621,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -634,7 +634,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -647,7 +647,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -674,29 +674,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -715,7 +715,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
@@ -748,24 +748,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -778,7 +778,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -791,7 +791,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -804,7 +804,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -831,29 +831,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -872,7 +872,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>

</xml_diff>

<commit_message>
2.3.4.dev1: Fix lazy loading and refactor indentation (#121)
</commit_message>
<xml_diff>
--- a/tests/data/dat.xlsx
+++ b/tests/data/dat.xlsx
@@ -22,16 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,26 +420,31 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.2" customWidth="1" min="1" max="1"/>
+    <col width="13.2" customWidth="1" min="2" max="2"/>
+    <col width="13.2" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -464,7 +457,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -477,7 +470,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -490,7 +483,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -515,31 +508,38 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.1" customWidth="1" min="1" max="1"/>
+    <col width="13.2" customWidth="1" min="2" max="2"/>
+    <col width="13.2" customWidth="1" min="3" max="3"/>
+    <col width="13.2" customWidth="1" min="4" max="4"/>
+    <col width="13.2" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -558,7 +558,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
@@ -591,24 +591,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -621,7 +621,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -634,7 +634,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -647,7 +647,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -674,29 +674,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -715,7 +715,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
@@ -748,24 +748,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
@@ -778,7 +778,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
@@ -791,7 +791,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
@@ -804,7 +804,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
@@ -831,29 +831,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Birmingham</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Manchester</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Leeds</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
@@ -872,7 +872,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>

</xml_diff>

<commit_message>
test(`store`): update test suite
</commit_message>
<xml_diff>
--- a/tests/data/dat.xlsx
+++ b/tests/data/dat.xlsx
@@ -421,9 +421,9 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.2" customWidth="1" min="1" max="1"/>
-    <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="13.2" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,11 +509,11 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.1" customWidth="1" min="1" max="1"/>
-    <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="13.2" customWidth="1" min="3" max="3"/>
-    <col width="13.2" customWidth="1" min="4" max="4"/>
-    <col width="13.2" customWidth="1" min="5" max="5"/>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +589,11 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -672,6 +677,13 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -746,6 +758,11 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -829,6 +846,13 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">

</xml_diff>

<commit_message>
Cleanup and refactoring (#130)
</commit_message>
<xml_diff>
--- a/tests/data/dat.xlsx
+++ b/tests/data/dat.xlsx
@@ -421,9 +421,9 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.2" customWidth="1" min="1" max="1"/>
-    <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="13.2" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,11 +509,11 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.1" customWidth="1" min="1" max="1"/>
-    <col width="13.2" customWidth="1" min="2" max="2"/>
-    <col width="13.2" customWidth="1" min="3" max="3"/>
-    <col width="13.2" customWidth="1" min="4" max="4"/>
-    <col width="13.2" customWidth="1" min="5" max="5"/>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +589,11 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -672,6 +677,13 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -746,6 +758,11 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.6" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -829,6 +846,13 @@
   </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.55" customWidth="1" min="1" max="1"/>
+    <col width="12.6" customWidth="1" min="2" max="2"/>
+    <col width="12.6" customWidth="1" min="3" max="3"/>
+    <col width="12.6" customWidth="1" min="4" max="4"/>
+    <col width="12.6" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">

</xml_diff>